<commit_message>
scan: seg7 2026-10-13 23:41 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-10-13.xlsx
+++ b/output/full_scan/batch_seq8_2026-10-13.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3389,21 +3389,21 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6947</v>
+        <v>7772</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>耀穎</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>454.8014528932949</v>
+        <v>458.0100505925537</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>125</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>46.28146313497048</v>
+        <v>40.8364816188262</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>11.48712870749814</v>
+        <v>42.53600070328574</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.396646432798511</v>
+        <v>0.5010050592553718</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.315647947164541</v>
+        <v>-7.401351303594414</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6862</v>
+        <v>6947</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>454.5700060032132</v>
+        <v>454.8014528932949</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>141.5</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,16 +3467,16 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.08793427002245</v>
+        <v>46.28146313497048</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>19.2219119629269</v>
+        <v>11.48712870749814</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.7925952403829392</v>
+        <v>1.396646432798511</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L57" s="2" t="n">
         <v>0</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>1.02308605669895</v>
+        <v>0.315647947164541</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3495,21 +3495,21 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>7732</v>
+        <v>6862</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>金興精密</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>445.4196870052128</v>
+        <v>454.5700060032132</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>33.55</v>
+        <v>141.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.46559181173139</v>
+        <v>51.08793427002245</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>6.686269203441929</v>
+        <v>19.2219119629269</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1.627036606717389</v>
+        <v>0.7925952403829392</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.6667682137464359</v>
+        <v>1.02308605669895</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>7788</v>
+        <v>7732</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>松川精密</t>
+          <t>金興精密</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>444.0199744977547</v>
+        <v>445.4196870052128</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>308.5</v>
+        <v>33.55</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>51.94663435871068</v>
+        <v>51.46559181173139</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>22.05209446926409</v>
+        <v>6.686269203441929</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.8484869865706053</v>
+        <v>1.627036606717389</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.1433895716927047</v>
+        <v>0.6667682137464359</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>7734</v>
+        <v>7788</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>印能科技</t>
+          <t>松川精密</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>443.429648541022</v>
+        <v>444.0199744977547</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>2700</v>
+        <v>308.5</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>47.24419130655276</v>
+        <v>51.94663435871068</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>14.23537188180277</v>
+        <v>22.05209446926409</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.499766580526803</v>
+        <v>0.8484869865706053</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>25.61541699987064</v>
+        <v>0.1433895716927047</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>7738</v>
+        <v>7734</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>東聯互動</t>
+          <t>印能科技</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>440.0845769733397</v>
+        <v>443.429648541022</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>157.5</v>
+        <v>2700</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>43.07139326006214</v>
+        <v>47.24419130655276</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>14.53991144157428</v>
+        <v>14.23537188180277</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.2038600836072137</v>
+        <v>1.499766580526803</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.588132303660521</v>
+        <v>25.61541699987064</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>7703</v>
+        <v>7738</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>銳澤</t>
+          <t>東聯互動</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>439.8475186292955</v>
+        <v>440.0845769733397</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>190</v>
+        <v>157.5</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>39.78418960180768</v>
+        <v>43.07139326006214</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>28.96648254773616</v>
+        <v>14.53991144157428</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2.49411254218928</v>
+        <v>0.2038600836072137</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-1.637199564892741</v>
+        <v>0.588132303660521</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6928</v>
+        <v>7703</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>銳澤</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>430.20857288872</v>
+        <v>439.8475186292955</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>45.1</v>
+        <v>190</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.71840879629121</v>
+        <v>39.78418960180768</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>13.74155047751233</v>
+        <v>28.96648254773616</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1.609338953050863</v>
+        <v>2.49411254218928</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.072420011404807</v>
+        <v>-1.637199564892741</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>7722</v>
+        <v>6928</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>LINEPAY</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>427.7126292526465</v>
+        <v>430.20857288872</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>261</v>
+        <v>45.1</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>43.16267051488574</v>
+        <v>44.71840879629121</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>14.68043772017962</v>
+        <v>13.74155047751233</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.8507048590281944</v>
+        <v>1.609338953050863</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>1.136078998440227</v>
+        <v>-0.072420011404807</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6859</v>
+        <v>7722</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>LINEPAY</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>422.012312955487</v>
+        <v>427.7126292526465</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>116</v>
+        <v>261</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>46.21949197197541</v>
+        <v>43.16267051488574</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>34.69964108808867</v>
+        <v>14.68043772017962</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.9298976022051016</v>
+        <v>0.8507048590281944</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>1</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.9155464275821212</v>
+        <v>1.136078998440227</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6840</v>
+        <v>6859</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>418.4630838606829</v>
+        <v>422.012312955487</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>85.90000000000001</v>
+        <v>116</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>35.69596065928179</v>
+        <v>46.21949197197541</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>26.32044689664625</v>
+        <v>34.69964108808867</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.8102788156499885</v>
+        <v>0.9298976022051016</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-2.195262169718704</v>
+        <v>-0.9155464275821212</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>7610</v>
+        <v>6840</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>聯友金屬-創</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>405.2402426564399</v>
+        <v>418.4630838606829</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>1545</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>38.22155703807833</v>
+        <v>35.69596065928179</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.10604509078614</v>
+        <v>26.32044689664625</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>1.042210113909899</v>
+        <v>0.8102788156499885</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-27.56139803594861</v>
+        <v>-2.195262169718704</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6890</v>
+        <v>7610</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>聯友金屬-創</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>399.2582219108536</v>
+        <v>405.2402426564399</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>149.5</v>
+        <v>1545</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>43.87168866406424</v>
+        <v>38.22155703807833</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>11.70237347995183</v>
+        <v>11.10604509078614</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>1.533285797183602</v>
+        <v>1.042210113909899</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>1.271899052473833</v>
+        <v>-27.56139803594861</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>7760</v>
+        <v>6890</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>399.170390289287</v>
+        <v>399.2582219108536</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>32.5</v>
+        <v>149.5</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>45.0524839646949</v>
+        <v>43.87168866406424</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>27.27044444098404</v>
+        <v>11.70237347995183</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>2.013865057879344</v>
+        <v>1.533285797183602</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>1</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0030098197490605</v>
+        <v>1.271899052473833</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6967</v>
+        <v>7760</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>394.3071763655758</v>
+        <v>399.170390289287</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>69.90000000000001</v>
+        <v>32.5</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>50.89303339650265</v>
+        <v>45.0524839646949</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>17.07765599148367</v>
+        <v>27.27044444098404</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.6174466400465232</v>
+        <v>2.013865057879344</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>1</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.4729724767362612</v>
+        <v>0.0030098197490605</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>7744</v>
+        <v>6967</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>崴寶</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>383.9727280751439</v>
+        <v>394.3071763655758</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>493</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>43.05186845662282</v>
+        <v>50.89303339650265</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>23.81531839590426</v>
+        <v>17.07765599148367</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1.192077034026476</v>
+        <v>0.6174466400465232</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-4.977171455213014</v>
+        <v>0.4729724767362612</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>7828</v>
+        <v>7744</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>創新服務</t>
+          <t>崴寶</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>382.4690535714183</v>
+        <v>383.9727280751439</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>1740</v>
+        <v>493</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>41.7775969482578</v>
+        <v>43.05186845662282</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>16.29335123236166</v>
+        <v>23.81531839590426</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1.146905357141831</v>
+        <v>1.192077034026476</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-26.36144318321625</v>
+        <v>-4.977171455213014</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>7818</v>
+        <v>7828</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>創新服務</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>374.5754939496917</v>
+        <v>382.4690535714183</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>59.8</v>
+        <v>1740</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>38.97715139732391</v>
+        <v>41.7775969482578</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.65769364962914</v>
+        <v>16.29335123236166</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.407535285036939</v>
+        <v>1.146905357141831</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.1353848078628101</v>
+        <v>-26.36144318321625</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>7736</v>
+        <v>7818</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>371.0935674884663</v>
+        <v>374.5754939496917</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>69</v>
+        <v>59.8</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>47.01585753994709</v>
+        <v>38.97715139732391</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>26.57597655906817</v>
+        <v>14.65769364962914</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.8188963201957821</v>
+        <v>0.407535285036939</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0543709046837136</v>
+        <v>0.1353848078628101</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>7856</v>
+        <v>7736</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>漢測</t>
+          <t>虎山</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>367.2297983222893</v>
+        <v>371.0935674884663</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>3800</v>
+        <v>69</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,49 +4421,49 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>35.7322661843146</v>
+        <v>47.01585753994709</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>13.16229493429142</v>
+        <v>26.57597655906817</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1.160260131235268</v>
+        <v>0.8188963201957821</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M75" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-89.92407823496326</v>
+        <v>0.0543709046837136</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>7740</v>
+        <v>7856</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>熙特爾-創</t>
+          <t>漢測</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>364.6775408752538</v>
+        <v>367.2297983222893</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>104.5</v>
+        <v>3800</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,49 +4474,49 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>38.45068554141776</v>
+        <v>35.7322661843146</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>25.2075650396832</v>
+        <v>13.16229493429142</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>1.272663615190865</v>
+        <v>1.160260131235268</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M76" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>1.04181272325443</v>
+        <v>-89.92407823496326</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6910</v>
+        <v>7740</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>德鴻</t>
+          <t>熙特爾-創</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>364.4768126877982</v>
+        <v>364.6775408752538</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>25.3</v>
+        <v>104.5</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>47.01925516449766</v>
+        <v>38.45068554141776</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>28.91638273175864</v>
+        <v>25.2075650396832</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.2218532049153105</v>
+        <v>1.272663615190865</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.097488504505872</v>
+        <v>1.04181272325443</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>7728</v>
+        <v>6910</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>德鴻</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>363.9685370802308</v>
+        <v>364.4768126877982</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>601</v>
+        <v>25.3</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>43.58875616744164</v>
+        <v>47.01925516449766</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>24.76894441394812</v>
+        <v>28.91638273175864</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.3313536089620554</v>
+        <v>0.2218532049153105</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-1.074761148726662</v>
+        <v>-0.097488504505872</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6907</v>
+        <v>7728</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>雅特力-KY</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>359.2425928891022</v>
+        <v>363.9685370802308</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>174</v>
+        <v>601</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>41.08113724899734</v>
+        <v>43.58875616744164</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>15.52112029249544</v>
+        <v>24.76894441394812</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.853366854654849</v>
+        <v>0.3313536089620554</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-1.29567097152443</v>
+        <v>-1.074761148726662</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>7805</v>
+        <v>6907</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>威聯通</t>
+          <t>雅特力-KY</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>355.8675124543283</v>
+        <v>359.2425928891022</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>475</v>
+        <v>174</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>33.26402485989509</v>
+        <v>41.08113724899734</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>26.27713159865698</v>
+        <v>15.52112029249544</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>2.428942803968652</v>
+        <v>0.853366854654849</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>2.974103776063497</v>
+        <v>-1.29567097152443</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>7791</v>
+        <v>7805</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>威聯通</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>349.0912418060965</v>
+        <v>355.8675124543283</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>51</v>
+        <v>475</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>19.27343633982812</v>
+        <v>33.26402485989509</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>27.45660964360597</v>
+        <v>26.27713159865698</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>4.252730566359422</v>
+        <v>2.428942803968652</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.2729141277598865</v>
+        <v>2.974103776063497</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4767,21 +4767,21 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6965</v>
+        <v>7791</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>346.8460039499723</v>
+        <v>349.0912418060965</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>66.59999999999999</v>
+        <v>51</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>46.43566932245469</v>
+        <v>19.27343633982812</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>43.91953295866973</v>
+        <v>27.45660964360597</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.8449604675097832</v>
+        <v>4.252730566359422</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.3607530445749849</v>
+        <v>-0.2729141277598865</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>8032</v>
+        <v>6965</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>344.0438356452983</v>
+        <v>346.8460039499723</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>34.8</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>36.94100545991409</v>
+        <v>46.43566932245469</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>14.25158245260762</v>
+        <v>43.91953295866973</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>1.851939020224806</v>
+        <v>0.8449604675097832</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.0170468474422887</v>
+        <v>0.3607530445749849</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6921</v>
+        <v>8032</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>343.8163522340215</v>
+        <v>344.0438356452983</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>64.90000000000001</v>
+        <v>34.8</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>51.49198389751805</v>
+        <v>36.94100545991409</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>17.87583093393734</v>
+        <v>14.25158245260762</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>3.227629153569714</v>
+        <v>1.851939020224806</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.2634225535261842</v>
+        <v>-0.0170468474422887</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6873</v>
+        <v>6921</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>340.3645912944301</v>
+        <v>343.8163522340215</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>65.09999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>36.73487862547834</v>
+        <v>51.49198389751805</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>15.62119078723263</v>
+        <v>17.87583093393734</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.8552269585049109</v>
+        <v>3.227629153569714</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.08794252398552491</v>
+        <v>-0.2634225535261842</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6923</v>
+        <v>6873</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>339.6740506166686</v>
+        <v>340.3645912944301</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>73.09999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,16 +5004,16 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>34.31205910416409</v>
+        <v>36.73487862547834</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.89738114431425</v>
+        <v>15.62119078723263</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>1.879484009865561</v>
+        <v>0.8552269585049109</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.2320156447075203</v>
+        <v>-0.08794252398552491</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6949</v>
+        <v>6923</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>沛爾生醫-創</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>335.3476164190521</v>
+        <v>339.6740506166686</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>42.05</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>25.6788166817628</v>
+        <v>34.31205910416409</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>45.59004997018672</v>
+        <v>12.89738114431425</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>1.259990739768259</v>
+        <v>1.879484009865561</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>32.50703736617749</v>
+        <v>-0.2320156447075203</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6958</v>
+        <v>6949</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>日盛台駿</t>
+          <t>沛爾生醫-創</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>334.6331298095748</v>
+        <v>335.3476164190521</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>16.95</v>
+        <v>42.05</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>45.40137020491581</v>
+        <v>25.6788166817628</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>20.60618706193061</v>
+        <v>45.59004997018672</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.3350886917960088</v>
+        <v>1.259990739768259</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.0328478942586218</v>
+        <v>32.50703736617749</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>7812</v>
+        <v>6958</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>稜研科技*-創</t>
+          <t>日盛台駿</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>330.8353126063218</v>
+        <v>334.6331298095748</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>63.9</v>
+        <v>16.95</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>30.8516637036888</v>
+        <v>45.40137020491581</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>24.23634573244908</v>
+        <v>20.60618706193061</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.4835312606321792</v>
+        <v>0.3350886917960088</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.6485668199993007</v>
+        <v>-0.0328478942586218</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5191,21 +5191,21 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6997</v>
+        <v>7812</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>博弘</t>
+          <t>稜研科技*-創</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>324.9926892147475</v>
+        <v>330.8353126063218</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>0</v>
+        <v>63.9</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>38.29830723437575</v>
+        <v>30.8516637036888</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>9.239444717026029</v>
+        <v>24.23634573244908</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.0022009464069549</v>
+        <v>0.4835312606321792</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-3.222683924960683</v>
+        <v>-0.6485668199993007</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>7547</v>
+        <v>6997</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>碩網</t>
+          <t>博弘</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>323.3799820343834</v>
+        <v>324.9926892147475</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>57.74859969610317</v>
+        <v>38.29830723437575</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>24.67379881658115</v>
+        <v>9.239444717026029</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.23799820343834</v>
+        <v>0.0022009464069549</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.0207193270566712</v>
+        <v>-3.222683924960683</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>7770</v>
+        <v>7547</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>碩網</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>317.2054570477513</v>
+        <v>323.3799820343834</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>39.45</v>
+        <v>59.5</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>50.24718251318579</v>
+        <v>57.74859969610317</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>13.11914797470873</v>
+        <v>24.67379881658115</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>1.092053537328819</v>
+        <v>0.23799820343834</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.2682270109930138</v>
+        <v>-0.0207193270566712</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6951</v>
+        <v>7770</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>君曜</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>314.8278093244191</v>
+        <v>317.2054570477513</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>68</v>
+        <v>39.45</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>26.26268607023971</v>
+        <v>50.24718251318579</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>32.63648710632047</v>
+        <v>13.11914797470873</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.7836423439043648</v>
+        <v>1.092053537328819</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.0619700385633767</v>
+        <v>-0.2682270109930138</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>7715</v>
+        <v>6951</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>裕山</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>312.9927404205836</v>
+        <v>314.8278093244191</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>26.8</v>
+        <v>68</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>36.72101262191632</v>
+        <v>26.26268607023971</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>22.74972344872304</v>
+        <v>32.63648710632047</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.7908470263175279</v>
+        <v>0.7836423439043648</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0141774549456467</v>
+        <v>-0.0619700385633767</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5456,21 +5456,21 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>7820</v>
+        <v>7715</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>立盈</t>
+          <t>裕山</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>311.526254667759</v>
+        <v>312.9927404205836</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>105</v>
+        <v>26.8</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>52.07048229390238</v>
+        <v>36.72101262191632</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>14.3855559108506</v>
+        <v>22.74972344872304</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.6554323507683474</v>
+        <v>0.7908470263175279</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-5.357763493242324</v>
+        <v>0.0141774549456467</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6895</v>
+        <v>7820</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>立盈</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>310.7210939944038</v>
+        <v>311.526254667759</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>151</v>
+        <v>105</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>53.5416920959601</v>
+        <v>52.07048229390238</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>14.91481295264873</v>
+        <v>14.3855559108506</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>1.029369668517776</v>
+        <v>0.6554323507683474</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0167075724228209</v>
+        <v>-5.357763493242324</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>7768</v>
+        <v>6895</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>309.7713661206462</v>
+        <v>310.7210939944038</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>283.5</v>
+        <v>151</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>45.38202854409857</v>
+        <v>53.5416920959601</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>24.96906252484258</v>
+        <v>14.91481295264873</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.8169048842355664</v>
+        <v>1.029369668517776</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.7867739028133336</v>
+        <v>0.0167075724228209</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>7749</v>
+        <v>7768</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>308.2274318707381</v>
+        <v>309.7713661206462</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>346</v>
+        <v>283.5</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>37.89622590037752</v>
+        <v>45.38202854409857</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>21.29402219930929</v>
+        <v>24.96906252484258</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.8944181564297609</v>
+        <v>0.8169048842355664</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-4.568572515334743</v>
+        <v>-0.7867739028133336</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8024</v>
+        <v>7749</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>305.84126585363</v>
+        <v>308.2274318707381</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>12.85</v>
+        <v>346</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>51.52689830286335</v>
+        <v>37.89622590037752</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>17.57016500707216</v>
+        <v>21.29402219930929</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.6382105578581172</v>
+        <v>0.8944181564297609</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.06868224402128301</v>
+        <v>-4.568572515334743</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8033</v>
+        <v>8024</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>雷虎</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>303.7919503631541</v>
+        <v>305.84126585363</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>164.5</v>
+        <v>12.85</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>38.18301283841267</v>
+        <v>51.52689830286335</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>8.05004824403148</v>
+        <v>17.57016500707216</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>1.029824787375895</v>
+        <v>0.6382105578581172</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.0613877008069176</v>
+        <v>0.06868224402128301</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6931</v>
+        <v>8033</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>青松健康</t>
+          <t>雷虎</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>301.188061974379</v>
+        <v>303.7919503631541</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>38</v>
+        <v>164.5</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>33.39795782394685</v>
+        <v>38.18301283841267</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>12.79779424516179</v>
+        <v>8.05004824403148</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>1.188860201524629</v>
+        <v>1.029824787375895</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0486609802921581</v>
+        <v>-0.0613877008069176</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>7750</v>
+        <v>6931</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>新代</t>
+          <t>青松健康</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>299.5553964270231</v>
+        <v>301.188061974379</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>1815</v>
+        <v>38</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,49 +5852,49 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>36.5137752237064</v>
+        <v>33.39795782394685</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>15.61920497704022</v>
+        <v>12.79779424516179</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.195744622123192</v>
+        <v>1.188860201524629</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L102" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M102" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>2.164493602271122</v>
+        <v>-0.0486609802921581</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>7780</v>
+        <v>7750</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>大研生醫*</t>
+          <t>新代</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>295.0189971969331</v>
+        <v>299.5553964270231</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>16.1</v>
+        <v>1815</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,49 +5905,49 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>45.27576550309819</v>
+        <v>36.5137752237064</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>18.41944817379032</v>
+        <v>15.61920497704022</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.7326660157671386</v>
+        <v>1.195744622123192</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M103" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.0406926079453535</v>
+        <v>2.164493602271122</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6887</v>
+        <v>7780</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>大研生醫*</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>293.4056704567232</v>
+        <v>295.0189971969331</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>35</v>
+        <v>16.1</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>35.25154632888321</v>
+        <v>45.27576550309819</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>32.09907096486421</v>
+        <v>18.41944817379032</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.585432351506223</v>
+        <v>0.7326660157671386</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.3511928820444601</v>
+        <v>0.0406926079453535</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6962</v>
+        <v>6887</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>奕力-KY</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>286.914590780457</v>
+        <v>293.4056704567232</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>31.8</v>
+        <v>35</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>47.48308292403816</v>
+        <v>35.25154632888321</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.8104830890156</v>
+        <v>32.09907096486421</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.7047807365867627</v>
+        <v>1.585432351506223</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0019811723141636</v>
+        <v>-0.3511928820444601</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>7689</v>
+        <v>6962</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>奕力-KY</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>286.7639291600639</v>
+        <v>286.914590780457</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>146.5</v>
+        <v>31.8</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>26.27028728710427</v>
+        <v>47.48308292403816</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>19.99863227533829</v>
+        <v>15.8104830890156</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>2.596332400240638</v>
+        <v>0.7047807365867627</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.1647682584117351</v>
+        <v>0.0019811723141636</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>7822</v>
+        <v>7689</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>倍利科</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>284.6619723204726</v>
+        <v>286.7639291600639</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>887</v>
+        <v>146.5</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>43.37966129589307</v>
+        <v>26.27028728710427</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.64471560063087</v>
+        <v>19.99863227533829</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1.339451101139978</v>
+        <v>2.596332400240638</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-2.184424399175409</v>
+        <v>-0.1647682584117351</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6996</v>
+        <v>7822</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>倍利科</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>282.0702821609818</v>
+        <v>284.6619723204726</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>165</v>
+        <v>887</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>37.62628174353595</v>
+        <v>43.37966129589307</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>18.40324029100181</v>
+        <v>17.64471560063087</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.88908831841548</v>
+        <v>1.339451101139978</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0945131989185275</v>
+        <v>-2.184424399175409</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6899</v>
+        <v>6996</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>278.6119187536636</v>
+        <v>282.0702821609818</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>49.1</v>
+        <v>165</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.60011145697077</v>
+        <v>37.62628174353595</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>24.0555331494335</v>
+        <v>18.40324029100181</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.266941414953678</v>
+        <v>0.88908831841548</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.013429697267084</v>
+        <v>-0.0945131989185275</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6919</v>
+        <v>6899</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>康霈*</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>278.5960863447603</v>
+        <v>278.6119187536636</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>76.5</v>
+        <v>49.1</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>31.45335936467657</v>
+        <v>42.60011145697077</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>30.10610215413426</v>
+        <v>24.0555331494335</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1.027993819248662</v>
+        <v>1.266941414953678</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.3934159607707403</v>
+        <v>0.013429697267084</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>7402</v>
+        <v>6919</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>康霈*</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>276.6939089010219</v>
+        <v>278.5960863447603</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>97.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,16 +6329,16 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>38.14962219349145</v>
+        <v>31.45335936467657</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>15.8360276679241</v>
+        <v>30.10610215413426</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.8073780462045628</v>
+        <v>1.027993819248662</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.1139942421054609</v>
+        <v>0.3934159607707403</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>7753</v>
+        <v>7402</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>261.8117228051413</v>
+        <v>276.6939089010219</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>35.6</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>41.81006736186306</v>
+        <v>38.14962219349145</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>9.650363394962609</v>
+        <v>15.8360276679241</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.9867367576753406</v>
+        <v>0.8073780462045628</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.09534912960526989</v>
+        <v>0.1139942421054609</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6410,21 +6410,21 @@
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6854</v>
+        <v>7753</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>261.6640353351589</v>
+        <v>261.8117228051413</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>90.8</v>
+        <v>35.6</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>45.05202542889123</v>
+        <v>41.81006736186306</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>13.13366759287153</v>
+        <v>9.650363394962609</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1.511337938011059</v>
+        <v>0.9867367576753406</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.1082290817409971</v>
+        <v>0.09534912960526989</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6908</v>
+        <v>6854</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>261.3330217987741</v>
+        <v>261.6640353351589</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>25.85</v>
+        <v>90.8</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>24.41435716805817</v>
+        <v>45.05202542889123</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>15.74166324912355</v>
+        <v>13.13366759287153</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.5313658087944098</v>
+        <v>1.511337938011059</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.1606478384329481</v>
+        <v>0.1082290817409971</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>7705</v>
+        <v>6908</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>三商餐飲</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>261.0455234007649</v>
+        <v>261.3330217987741</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>29.45</v>
+        <v>25.85</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>34.74600487677947</v>
+        <v>24.41435716805817</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>9.771301565738661</v>
+        <v>15.74166324912355</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.421230611555558</v>
+        <v>0.5313658087944098</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0137121843748325</v>
+        <v>-0.1606478384329481</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6569,21 +6569,21 @@
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6994</v>
+        <v>7705</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>富威電力</t>
+          <t>三商餐飲</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>243.8829401116557</v>
+        <v>261.0455234007649</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>28.3</v>
+        <v>29.45</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>40.32041213564221</v>
+        <v>34.74600487677947</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>30.51321866606477</v>
+        <v>9.771301565738661</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6525199948797317</v>
+        <v>1.421230611555558</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.4156994614951166</v>
+        <v>-0.0137121843748325</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>7823</v>
+        <v>6994</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>奧義賽博-KY創</t>
+          <t>富威電力</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>236.9523987414797</v>
+        <v>243.8829401116557</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>78.2</v>
+        <v>28.3</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>38.84391623491212</v>
+        <v>40.32041213564221</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>13.93737064006763</v>
+        <v>30.51321866606477</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.5346637279525249</v>
+        <v>0.6525199948797317</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.0744285345487101</v>
+        <v>0.4156994614951166</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6906</v>
+        <v>7823</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>奧義賽博-KY創</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>236.4502053053816</v>
+        <v>236.9523987414797</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>78.5</v>
+        <v>78.2</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>44.03555842855254</v>
+        <v>38.84391623491212</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>31.46823773928907</v>
+        <v>13.93737064006763</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.4199925465623185</v>
+        <v>0.5346637279525249</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.8014530010739552</v>
+        <v>-0.0744285345487101</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>7721</v>
+        <v>6906</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>226.7063930733576</v>
+        <v>236.4502053053816</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>60.4</v>
+        <v>78.5</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>43.95659688434853</v>
+        <v>44.03555842855254</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>20.0698781801268</v>
+        <v>31.46823773928907</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.6940742201809011</v>
+        <v>0.4199925465623185</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.07947218238876939</v>
+        <v>-0.8014530010739552</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6781,21 +6781,21 @@
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6969</v>
+        <v>7721</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>成信實業*-創</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>194.3786383544988</v>
+        <v>226.7063930733576</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>29.5</v>
+        <v>60.4</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>38.03572844678418</v>
+        <v>43.95659688434853</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>11.10697323420356</v>
+        <v>20.0698781801268</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.9201122143400288</v>
+        <v>0.6940742201809011</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.1935627075262838</v>
+        <v>-0.07947218238876939</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>7786</v>
+        <v>6969</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>東方風能</t>
+          <t>成信實業*-創</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>179.357375686266</v>
+        <v>194.3786383544988</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>116</v>
+        <v>29.5</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>44.13513855864303</v>
+        <v>38.03572844678418</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>11.58033409903129</v>
+        <v>11.10697323420356</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.046424202822671</v>
+        <v>0.9201122143400288</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.1190651505261793</v>
+        <v>-0.1935627075262838</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>7803</v>
+        <v>7786</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>雲象科技-創</t>
+          <t>東方風能</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>176.6508484846414</v>
+        <v>179.357375686266</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>16.2</v>
+        <v>116</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,16 +6912,16 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>22.60260338299764</v>
+        <v>44.13513855864303</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>21.20159487327934</v>
+        <v>11.58033409903129</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>1.06508484846414</v>
+        <v>1.046424202822671</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.1206761561010221</v>
+        <v>-0.1190651505261793</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>8034</v>
+        <v>7803</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>榮群</t>
+          <t>雲象科技-創</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>174.288054936666</v>
+        <v>176.6508484846414</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>19.1</v>
+        <v>16.2</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>38.21581963208867</v>
+        <v>22.60260338299764</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15.92415464701511</v>
+        <v>21.20159487327934</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.8144242097787058</v>
+        <v>1.06508484846414</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.1397298004055152</v>
+        <v>-0.1206761561010221</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6865</v>
+        <v>8034</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>偉康科技</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>171.6459560757339</v>
+        <v>174.288054936666</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>0</v>
+        <v>19.1</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>15.92514205680808</v>
+        <v>38.21581963208867</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.26809912037358</v>
+        <v>15.92415464701511</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.0054236289434302</v>
+        <v>0.8144242097787058</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-2.037337238346314</v>
+        <v>-0.1397298004055152</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>7825</v>
+        <v>6865</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>和亞智慧</t>
+          <t>偉康科技</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>166.921156757875</v>
+        <v>171.6459560757339</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>70.8</v>
+        <v>0</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>38.09465813597082</v>
+        <v>15.92514205680808</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>15.75183325536592</v>
+        <v>17.26809912037358</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.3144623351506075</v>
+        <v>0.0054236289434302</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,62 +7089,115 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.295470806548592</v>
+        <v>-2.037337238346314</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
+        <v>7825</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>和亞智慧</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>166.921156757875</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>38.09465813597082</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>15.75183325536592</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.3144623351506075</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>-1.295470806548592</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
         <v>6855</v>
       </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>數泓科</t>
         </is>
       </c>
-      <c r="C126" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D126" s="2" t="n">
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>161.9499182293609</v>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E127" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2" t="n">
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>52.06343485221353</v>
       </c>
-      <c r="I126" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>7.649660555912372</v>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J127" s="2" t="n">
         <v>0.7314484222715431</v>
       </c>
-      <c r="K126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N126" s="2" t="n">
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
         <v>5.032279012327164</v>
       </c>
-      <c r="O126" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>

</xml_diff>

<commit_message>
scan: seg7 2026-10-14 00:58 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-10-13.xlsx
+++ b/output/full_scan/batch_seq8_2026-10-13.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>73.21451432935567</v>
+        <v>73.21451436462419</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>32.97049002986571</v>
+        <v>32.97049000816322</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>6.40126400459638</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.183672951359434</v>
+        <v>1.183672950998931</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>68.68797140011094</v>
+        <v>68.68797148782357</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>37.23522848951056</v>
+        <v>37.23522868084014</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>3.647117664407341</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.830859292421338</v>
+        <v>2.830859291339799</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>74.43351296662445</v>
+        <v>74.43351345123632</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>44.407542251672</v>
+        <v>44.40754327264069</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>3.334706372876469</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1.029990618978614</v>
+        <v>1.029990616695329</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>57.5102951317587</v>
+        <v>57.51029512146997</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>13.83199830581685</v>
+        <v>13.83199815499223</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.032096120049246</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>12.10477839262433</v>
+        <v>12.10477839430684</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>910.234880102986</v>
+        <v>910.2348801029846</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>143</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>62.28326766589954</v>
+        <v>62.28326796392723</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>19.09091577565949</v>
+        <v>19.0909158037218</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>6.727674196847715</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1.841113625166417</v>
+        <v>1.841113623964681</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>57.64162725873858</v>
+        <v>57.64162732278032</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>12.45702543823285</v>
+        <v>12.45702560361794</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.732596966854401</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.555384429016257</v>
+        <v>1.555384428655734</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>54.64875568924279</v>
+        <v>54.64875572566346</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>31.91743564740131</v>
+        <v>31.91743570543387</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.871291255746362</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-0.1917669770438559</v>
+        <v>-0.1917669778850532</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>61.7273889914181</v>
+        <v>61.7273890297406</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>46.76802066108277</v>
+        <v>46.76802076955785</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.857541148226222</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-3.203833724894594</v>
+        <v>-3.20383372609632</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>51.92808492893351</v>
+        <v>51.92808491864428</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>15.13207924228231</v>
+        <v>15.13207926284878</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.7941479116646</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.4068869610804086</v>
+        <v>0.4068869608400591</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>712.9542793228366</v>
+        <v>712.9542793228364</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>276</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>56.14711788373689</v>
+        <v>56.14711796727158</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>28.54342001912111</v>
+        <v>28.54342015870558</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.5001415006928642</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>1.504146385065002</v>
+        <v>1.504146384223826</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>44.94603088070998</v>
+        <v>44.94603108320109</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>22.44705573774336</v>
+        <v>22.4470558217769</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.622071282821222</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.08145783532193671</v>
+        <v>-0.0814578367639946</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57.16878817257633</v>
+        <v>57.16878821078098</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>51.11213607526474</v>
+        <v>51.11213609898274</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.6792340017800361</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-3.871233236581333</v>
+        <v>-3.871233237422558</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.70298522582802</v>
+        <v>60.70298539880021</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>25.67610320366269</v>
+        <v>25.67610343914079</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.644767291097026</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.1172886913569677</v>
+        <v>0.1172886912608303</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>53.81767840389403</v>
+        <v>53.81767841913705</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>48.13972815853</v>
+        <v>48.13972816422573</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.4852034510569841</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.4603081667217719</v>
+        <v>-0.4603081666376512</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>666.0441355265576</v>
+        <v>666.0441355265583</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>805</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>55.19356721167822</v>
+        <v>55.19356726047275</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>32.61261117601315</v>
+        <v>32.61261123268766</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.119134885165447</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>9.801723505411619</v>
+        <v>9.801723504930925</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>641.1729773454597</v>
+        <v>641.1729773454612</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>6070</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>50.55382498086355</v>
+        <v>50.5538249763813</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>14.176537281815</v>
+        <v>14.17653722170694</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.8077671326760562</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>54.12166023876192</v>
+        <v>54.12166025318309</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>60.90555547862512</v>
+        <v>60.90555584572498</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>20.08438072620697</v>
+        <v>20.08438072694154</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.2298113379521614</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.1335095430350597</v>
+        <v>0.1335095427105917</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51.48540834533637</v>
+        <v>51.48540836590081</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>20.65857672605877</v>
+        <v>20.65857687733722</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.5433342008849026</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>2.171131831377741</v>
+        <v>2.171131830897075</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>61.43476786091863</v>
+        <v>61.43476805023376</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>35.34986592352274</v>
+        <v>35.34986605982637</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.8162083282292315</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>1.83899389159</v>
+        <v>1.838993888946156</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>50.59670346211978</v>
+        <v>50.5967034739434</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>31.66463043336697</v>
+        <v>31.66463048276364</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.8516205873184823</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-2.773283956074525</v>
+        <v>-2.773283956435055</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>56.23937436758286</v>
+        <v>56.23937398261432</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>24.10020298065393</v>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>587.2562623875502</v>
+        <v>587.2562623875506</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>16.55</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>57.34220770223404</v>
+        <v>57.3422080692775</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>30.59125498285703</v>
+        <v>30.59125493323121</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.542855052116946</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.0802776374246837</v>
+        <v>0.0802776372203894</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>51.09406597607365</v>
+        <v>51.09406601129233</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>17.14762289878232</v>
+        <v>17.14762303982479</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.3162493078200947</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0067567772703925</v>
+        <v>0.0067567770540763</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>585.9602979080286</v>
+        <v>585.960297908028</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>323</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>54.97385216281265</v>
+        <v>54.97385218915623</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>20.63904695415376</v>
+        <v>20.63904696253333</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.232588405904882</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>2.673861071965236</v>
+        <v>2.673861072205581</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>53.21911710839223</v>
+        <v>53.21911718844908</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>35.03286733955341</v>
+        <v>35.0328672449665</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.466399763583973</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.2019890737969527</v>
+        <v>-0.2019890740372876</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>572.4095999483619</v>
+        <v>572.4095999483618</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>75</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>52.07339464885748</v>
+        <v>52.07339489715729</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>31.66753005430537</v>
+        <v>31.66753016588729</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.3676344561952028</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.1004615724101229</v>
+        <v>0.1004615720736323</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>554.5111373977772</v>
+        <v>554.5111373977776</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>36.3</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>41.59576776302434</v>
+        <v>41.59576779975527</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>33.17129227599273</v>
+        <v>33.17129227407948</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.7762641723439082</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0329087771814931</v>
+        <v>0.0329087770733338</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>50.60781674895811</v>
+        <v>50.60781683925062</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>22.95994793098146</v>
+        <v>22.95994798279881</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.097814773521598</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>1.094038581710152</v>
+        <v>1.094038581349632</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>54.32887544254182</v>
+        <v>54.32887556310857</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>32.25240258053334</v>
+        <v>32.25240253669894</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.2784215697705736</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-0.4315187816222186</v>
+        <v>-0.4315187817424029</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>550.4209087760905</v>
+        <v>550.4209087760906</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>163</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>51.29590648308549</v>
+        <v>51.29590646600877</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>30.5484798149626</v>
+        <v>30.54847993368176</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.9751688986559102</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0207414127822032</v>
+        <v>0.0207414132629253</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>52.70808982590129</v>
+        <v>52.70808994021775</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>22.91679334558706</v>
+        <v>22.91679346858875</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.4708951073579023</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.2014983631343687</v>
+        <v>0.2014983624133322</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>547.3506683655792</v>
+        <v>547.3506683655812</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>139</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>59.28427086975321</v>
+        <v>59.28427094922688</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>22.31984335559983</v>
+        <v>22.31984336128769</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.901708721315143</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.099878501213924</v>
+        <v>1.099878500060265</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.03703892173093</v>
+        <v>52.03703897912602</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>31.3533480923939</v>
+        <v>31.35334811986828</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.210924594055553</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-1.084233121838267</v>
+        <v>-1.084233122799652</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>51.15626795358681</v>
+        <v>51.15626796496925</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>36.99502111114572</v>
+        <v>36.99502113512456</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.4202365633669098</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-2.747165465960713</v>
+        <v>-2.74716546634523</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>52.49706926337816</v>
+        <v>52.49706924732257</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>29.93671326311685</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.541695312987903</v>
+        <v>0.5416953134686029</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>60.79482031182199</v>
+        <v>60.79482048425676</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>29.14764898068863</v>
+        <v>29.14764902465104</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>5.905577978843622</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.4336342352023193</v>
+        <v>0.4336342349379403</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>525.9286252076949</v>
+        <v>525.9286252076948</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>163.5</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>54.05626970999798</v>
+        <v>54.05626989843508</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>16.96841194146156</v>
+        <v>16.96841209996549</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.8554305940406706</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.2632021354983642</v>
+        <v>0.2632021353301272</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>29.4903648523847</v>
+        <v>29.49036500074658</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>35.43732487835707</v>
+        <v>35.43732493776021</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>1.968456755850453</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.6132187208817776</v>
+        <v>0.6132187204010799</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>47.04963992365672</v>
+        <v>47.04963975929719</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>19.27297086071457</v>
+        <v>19.27297086620129</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4734232315503106</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-1.230854120874374</v>
+        <v>-1.230854120994535</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>55.15786481861383</v>
+        <v>55.15786492301731</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>31.72130274399066</v>
+        <v>31.72130274399065</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.5318573610692862</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.0466903590799627</v>
+        <v>-0.0466903591280302</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>47.77099333563481</v>
+        <v>47.77099346566763</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>25.95275345825714</v>
+        <v>25.95275360897444</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.5484328189121633</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-2.285631295018277</v>
+        <v>-2.285631296941021</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>514.0378397226712</v>
+        <v>514.0378397226716</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>32.4</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>56.89576365297002</v>
+        <v>56.89576361358444</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>15.09900710809162</v>
+        <v>15.099007124253</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.65703768709473</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.07090447863268109</v>
+        <v>0.07090447869276879</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>511.5619275176673</v>
+        <v>511.5619275176672</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>39</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.15777540258407</v>
+        <v>52.15777540523213</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>8.157424410426541</v>
+        <v>8.157424445054172</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>3.07775275610625</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.4269359807702546</v>
+        <v>0.426935980722181</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>501.7674247802061</v>
+        <v>501.767424780206</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>24.6</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>52.12677471969699</v>
+        <v>52.1267747074909</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>25.51921204048318</v>
+        <v>25.519212149922</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.6108785425674623</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.1593751628135945</v>
+        <v>0.1593751628256097</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>500.1887473812226</v>
+        <v>500.1887473812225</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>17.5</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>58.50846260534123</v>
+        <v>58.50846270452627</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>29.63086855698357</v>
+        <v>29.63086862073415</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.04234198019281</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.2006890703739328</v>
+        <v>0.2006890703138432</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>46.33820722181598</v>
+        <v>46.33820723802512</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>23.5911985690343</v>
+        <v>23.59119862279269</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.8800960648763188</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-2.878368284512502</v>
+        <v>-2.878368284704792</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>50.35020627577948</v>
+        <v>50.3502063153366</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>23.68788884421014</v>
+        <v>23.68788889723134</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5046538886354175</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>48.40820908835913</v>
+        <v>48.40820910867948</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>5.37531532865578</v>
+        <v>5.375315328150331</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.9153978476279836</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.6604698364418344</v>
+        <v>0.6604698363216572</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>483.5536869726631</v>
+        <v>483.5536869726632</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>111</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>51.654007808575</v>
+        <v>51.65400781883113</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>7.08070572501722</v>
+        <v>7.080705693051302</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.029477575509538</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.8450498502246545</v>
+        <v>0.8450498496238039</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>482.2760002684195</v>
+        <v>482.2760002684192</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>80</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>63.39318027603351</v>
+        <v>63.39318032180631</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>17.84353906003615</v>
+        <v>17.84353907291614</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>2.42380753934851</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.5098759245882936</v>
+        <v>0.5098759244200592</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>53.41787223805311</v>
+        <v>53.41787217531235</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>20.50511558268294</v>
+        <v>20.50511557781555</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.789022732188423</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.07563690965721941</v>
+        <v>0.07563690953703919</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>47.54179050865569</v>
+        <v>47.54179063123635</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>40.85028964273817</v>
+        <v>40.85028962486194</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1.033062258455309</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-8.219577229046635</v>
+        <v>-8.219577231930792</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.28146313497048</v>
+        <v>46.28146322211244</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>11.48712870749814</v>
+        <v>11.4871289046523</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.396646432798511</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.315647947164541</v>
+        <v>0.3156479469722681</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>454.5700060032132</v>
+        <v>454.5700060032119</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>141.5</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.08793427002245</v>
+        <v>51.08793431449767</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>19.2219119629269</v>
+        <v>19.22191201700565</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.7925952403829392</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>1.02308605669895</v>
+        <v>1.023086056458598</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>51.46559181173139</v>
+        <v>51.46559181101351</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>6.686269203441929</v>
+        <v>6.686269222890664</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.627036606717389</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.6667682137464359</v>
+        <v>0.6667682137704714</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,7 +3626,7 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>51.94663435871068</v>
+        <v>51.94663437642502</v>
       </c>
       <c r="I60" s="2" t="n">
         <v>22.05209446926409</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.1433895716927047</v>
+        <v>0.1433895714523281</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>443.429648541022</v>
+        <v>443.4296485410221</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>2700</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>47.24419130655276</v>
+        <v>47.24419132826515</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>14.23537188180277</v>
+        <v>14.23537197565073</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.499766580526803</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>25.61541699987064</v>
+        <v>25.61541699025685</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>440.0845769733397</v>
+        <v>440.0845769733388</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>157.5</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>43.07139326006214</v>
+        <v>43.07139355123291</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>14.53991144157428</v>
+        <v>14.53991143202422</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.2038600836072137</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.588132303660521</v>
+        <v>0.5881323029394929</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>39.78418960180768</v>
+        <v>39.78418954329938</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>28.96648254773616</v>
+        <v>28.96648252409538</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>2.49411254218928</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-1.637199564892741</v>
+        <v>-1.637199565133102</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>44.71840879629121</v>
+        <v>44.71840918416381</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>13.74155047751233</v>
+        <v>13.74155077476193</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1.609338953050863</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.072420011404807</v>
+        <v>-0.07242001255846831</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>43.16267051488574</v>
+        <v>43.16267157122266</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>14.68043772017962</v>
+        <v>14.68043760033742</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.8507048590281944</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>1.136078998440227</v>
+        <v>1.136078992191246</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>422.012312955487</v>
+        <v>422.0123129554871</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>116</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>46.21949197197541</v>
+        <v>46.21949223811239</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>34.69964108808867</v>
+        <v>34.69964117947509</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.9298976022051016</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.9155464275821212</v>
+        <v>-0.915546428543518</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>35.69596065928179</v>
+        <v>35.69596070260468</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>26.32044689664625</v>
+        <v>26.32044690097073</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.8102788156499885</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-2.195262169718704</v>
+        <v>-2.195262169935007</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>38.22155703807833</v>
+        <v>38.22155703707448</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>11.10604509078614</v>
+        <v>11.10604505229487</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.042210113909899</v>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>399.2582219108536</v>
+        <v>399.2582219108535</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>149.5</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>43.87168866406424</v>
+        <v>43.87168865002262</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>11.70237347995183</v>
+        <v>11.70237351348454</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.533285797183602</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>1.271899052473833</v>
+        <v>1.271899053194895</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>399.170390289287</v>
+        <v>399.1703902892868</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>32.5</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0030098197490605</v>
+        <v>0.0030098197610792</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>50.89303339650265</v>
+        <v>50.89303352383624</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>17.07765599148367</v>
+        <v>17.07765611919841</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6174466400465232</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.4729724767362612</v>
+        <v>0.4729724763517113</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>43.05186845662282</v>
+        <v>43.05186848517541</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>23.81531839590426</v>
+        <v>23.8153184660806</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>1.192077034026476</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-4.977171455213014</v>
+        <v>-4.9771714560543</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>41.7775969482578</v>
+        <v>41.77759695554119</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>16.29335123236166</v>
+        <v>16.29335124204896</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>1.146905357141831</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-26.36144318321625</v>
+        <v>-26.36144318586003</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>38.97715139732391</v>
+        <v>38.97715262280904</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.65769364962914</v>
+        <v>14.65769363565433</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.407535285036939</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.1353848078628101</v>
+        <v>0.1353848077426417</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>371.0935674884663</v>
+        <v>371.0935674884668</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>69</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>47.01585753994709</v>
+        <v>47.01585763569559</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>26.57597655906817</v>
+        <v>26.57597672684559</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.8188963201957821</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0543709046837136</v>
+        <v>0.0543709043953074</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>38.45068554141776</v>
+        <v>38.45068564247005</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>25.2075650396832</v>
+        <v>25.20756511543795</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1.272663615190865</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>1.04181272325443</v>
+        <v>1.041812721091327</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>364.4768126877982</v>
+        <v>364.4768126877975</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>25.3</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>47.01925516449766</v>
+        <v>47.01925635194484</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>28.91638273175864</v>
+        <v>28.91638269229558</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.2218532049153105</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.097488504505872</v>
+        <v>-0.09748850452990809</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4636,7 +4636,7 @@
         <v>43.58875616744164</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>24.76894441394812</v>
+        <v>24.76894446431722</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.3313536089620554</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-1.074761148726662</v>
+        <v>-1.074761149327546</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>33.26402485989509</v>
+        <v>33.26402495588191</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>26.27713159865698</v>
+        <v>26.27713162749155</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>2.428942803968652</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>2.974103776063497</v>
+        <v>2.974103773900442</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>349.0912418060965</v>
+        <v>349.0912418060967</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>51</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>19.27343633982812</v>
+        <v>19.27343638603543</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.45660964360597</v>
+        <v>27.45660960049243</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>4.252730566359422</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.2729141277598865</v>
+        <v>-0.2729141280002312</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>46.43566932245469</v>
+        <v>46.43566936816198</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>43.91953295866973</v>
+        <v>43.91953296238941</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.8449604675097832</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.3607530445749849</v>
+        <v>0.3607530443586646</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>344.0438356452983</v>
+        <v>344.0438356452985</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>34.8</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>36.94100545991409</v>
+        <v>36.94100616993549</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>14.25158245260762</v>
+        <v>14.25158260351905</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.851939020224806</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0170468474422887</v>
+        <v>-0.017046847922978</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>36.73487862547834</v>
+        <v>36.73487899912489</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>15.62119078723263</v>
+        <v>15.62119075080009</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.8552269585049109</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.08794252398552491</v>
+        <v>-0.0879425248267451</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>339.6740506166686</v>
+        <v>339.674050616662</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>73.09999999999999</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>34.31205910416409</v>
+        <v>34.31206062200961</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>12.89738114431425</v>
+        <v>12.89738108737498</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.879484009865561</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>25.6788166817628</v>
+        <v>25.67881674742939</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>45.59004997018672</v>
+        <v>45.59005003131668</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.259990739768259</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>32.50703736617749</v>
+        <v>32.50703736411793</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>45.40137020491581</v>
+        <v>45.40137015927933</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>20.60618706193061</v>
+        <v>20.60618725360917</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.3350886917960088</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>30.8516637036888</v>
+        <v>30.8516637272788</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>24.23634573244908</v>
+        <v>24.23634604605252</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.4835312606321792</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.6485668199993007</v>
+        <v>-0.6485668203838522</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>38.29830723437575</v>
+        <v>38.29830722884916</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>9.239444717026029</v>
+        <v>9.239444759853168</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.0022009464069549</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-3.222683924960683</v>
+        <v>-3.22268392472033</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>57.74859969610317</v>
+        <v>57.748599808107</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>24.67379881658115</v>
+        <v>24.67379881004837</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.23799820343834</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0207193270566712</v>
+        <v>-0.0207193275373622</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>317.2054570477513</v>
+        <v>317.2054570477509</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>39.45</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>50.24718251318579</v>
+        <v>50.24718256307322</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>13.11914797470873</v>
+        <v>13.11914780491427</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.092053537328819</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.2682270109930138</v>
+        <v>-0.268227011065115</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>26.26268607023971</v>
+        <v>26.26268640963828</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>32.63648710632047</v>
+        <v>32.63648704413669</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.7836423439043648</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.0619700385633767</v>
+        <v>-0.0619700386354746</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>312.9927404205836</v>
+        <v>312.9927404205831</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>26.8</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>36.72101262191632</v>
+        <v>36.72101245648565</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>22.74972344872304</v>
+        <v>22.74972339411764</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.7908470263175279</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0141774549456467</v>
+        <v>0.0141774548134578</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>311.526254667759</v>
+        <v>311.5262546677617</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>105</v>
@@ -5534,7 +5534,7 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>52.07048229390238</v>
+        <v>52.07048234973737</v>
       </c>
       <c r="I96" s="2" t="n">
         <v>14.3855559108506</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-5.357763493242324</v>
+        <v>-5.35776349624664</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>53.5416920959601</v>
+        <v>53.54169242029917</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.91481295264873</v>
+        <v>14.91481299818401</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.029369668517776</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0167075724228209</v>
+        <v>0.0167075708605892</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>45.38202854409857</v>
+        <v>45.38202853531376</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>24.96906252484258</v>
+        <v>24.96906257445419</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.8169048842355664</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.7867739028133336</v>
+        <v>-0.7867739032939696</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>37.89622590037752</v>
+        <v>37.89622639748727</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>21.29402219930929</v>
+        <v>21.29402221248889</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.8944181564297609</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-4.568572515334743</v>
+        <v>-4.5685725261503</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>305.84126585363</v>
+        <v>305.8412658536301</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>12.85</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>51.52689830286335</v>
+        <v>51.52689845837268</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>17.57016500707216</v>
+        <v>17.5701649582514</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.6382105578581172</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.06868224402128301</v>
+        <v>0.06868224396119441</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>38.18301283841267</v>
+        <v>38.18301303044965</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>8.05004824403148</v>
+        <v>8.050048547317688</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>1.029824787375895</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0613877008069176</v>
+        <v>-0.0613877015279626</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>301.188061974379</v>
+        <v>301.1880619743789</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>38</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>33.39795782394685</v>
+        <v>33.39795787522264</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>12.79779424516179</v>
+        <v>12.7977943684632</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.188860201524629</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0486609802921581</v>
+        <v>-0.0486609802801407</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>299.5553964270231</v>
+        <v>299.5553964270226</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>1815</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>36.5137752237064</v>
+        <v>36.5137752320679</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>15.61920497704022</v>
+        <v>15.61920505047286</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>1.195744622123192</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>2.164493602271122</v>
+        <v>2.164493599146724</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>45.27576550309819</v>
+        <v>45.27576094350791</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>18.41944817379032</v>
+        <v>18.41944708782771</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.7326660157671386</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.0406926079453535</v>
+        <v>0.040692607182556</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>293.4056704567232</v>
+        <v>293.405670456714</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>35</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>35.25154632888321</v>
+        <v>35.25154626225392</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>32.09907096486421</v>
+        <v>32.09907091114877</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.585432351506223</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.3511928820444601</v>
+        <v>-0.3511928820204273</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>47.48308292403816</v>
+        <v>47.48308317333733</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>15.8104830890156</v>
+        <v>15.81048313255649</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7047807365867627</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0019811723141636</v>
+        <v>0.0019811721338965</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>284.6619723204726</v>
+        <v>284.6619723204728</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>887</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>43.37966129589307</v>
+        <v>43.37966149021207</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>17.64471560063087</v>
+        <v>17.6447158041702</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.339451101139978</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-2.184424399175409</v>
+        <v>-2.184424404222732</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>282.0702821609818</v>
+        <v>282.0702821609798</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>165</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>37.62628174353595</v>
+        <v>37.62628190502304</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.40324029100181</v>
+        <v>18.4032405756898</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.88908831841548</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.0945131989185275</v>
+        <v>-0.09451319987990291</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>278.6119187536636</v>
+        <v>278.6119187536795</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>49.1</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>42.60011145697077</v>
+        <v>42.60011146678301</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>24.0555331494335</v>
+        <v>24.05553318674993</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.266941414953678</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.013429697267084</v>
+        <v>0.013429697327172</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>31.45335936467657</v>
+        <v>31.4533602473902</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>30.10610215413426</v>
+        <v>30.10610222456952</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>1.027993819248662</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.3934159607707403</v>
+        <v>0.3934159613716161</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>276.6939089010219</v>
+        <v>276.6939089010217</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>97.90000000000001</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>38.14962219349145</v>
+        <v>38.14962231916611</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>15.8360276679241</v>
+        <v>15.83602769241935</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.8073780462045628</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1139942421054609</v>
+        <v>0.1139942420333592</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>41.81006736186306</v>
+        <v>41.81006841720016</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>9.650363394962609</v>
+        <v>9.650363352663902</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.9867367576753406</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.09534912960526989</v>
+        <v>0.09534912922071941</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>261.6640353351589</v>
+        <v>261.664035335159</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>90.8</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.05202542889123</v>
+        <v>45.05202600964095</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>13.13366759287153</v>
+        <v>13.13366760036533</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.511337938011059</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.1082290817409971</v>
+        <v>0.1082290802989304</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>24.41435716805817</v>
+        <v>24.41435695463113</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>15.74166324912355</v>
+        <v>15.7416631586715</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.5313658087944098</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1606478384329481</v>
+        <v>-0.1606478382166376</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>261.0455234007649</v>
+        <v>261.0455234007652</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>29.45</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>34.74600487677947</v>
+        <v>34.74600474110841</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>9.771301565738661</v>
+        <v>9.771301729819941</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>1.421230611555558</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.0137121843748325</v>
+        <v>-0.0137121843027261</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>40.32041213564221</v>
+        <v>40.32041232421261</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>30.51321866606477</v>
+        <v>30.5132185648393</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.6525199948797317</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.4156994614951166</v>
+        <v>0.4156994608942495</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>44.03555842855254</v>
+        <v>44.03555858372638</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>31.46823773928907</v>
+        <v>31.46823773744005</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.4199925465623185</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.8014530010739552</v>
+        <v>-0.8014530011941171</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>43.95659688434853</v>
+        <v>43.95659716294306</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>20.0698781801268</v>
+        <v>20.06987844375953</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.6940742201809011</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.07947218238876939</v>
+        <v>-0.07947218284542749</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>38.03572844678418</v>
+        <v>38.03572862513707</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>11.10697323420356</v>
+        <v>11.10697339913305</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.9201122143400288</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.1935627075262838</v>
+        <v>-0.1935627081391673</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>179.357375686266</v>
+        <v>179.3573756862659</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>116</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>44.13513855864303</v>
+        <v>44.13513901363227</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>11.58033409903129</v>
+        <v>11.58033407959646</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.046424202822671</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.1190651505261793</v>
+        <v>-0.1190651525691215</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>22.60260338299764</v>
+        <v>22.60260314581549</v>
       </c>
       <c r="I123" s="2" t="n">
         <v>21.20159487327934</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.1206761561010221</v>
+        <v>-0.1206761559207632</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>174.288054936666</v>
+        <v>174.2880549366819</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>19.1</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>38.21581963208867</v>
+        <v>38.21581966561417</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.92415464701511</v>
+        <v>15.92415479358958</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.8144242097787058</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.1397298004055152</v>
+        <v>-0.1397298003694636</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>15.92514205680808</v>
+        <v>15.92514205330957</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.26809912037358</v>
+        <v>17.26809919006451</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.0054236289434302</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-2.037337238346314</v>
+        <v>-2.037337238418419</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>38.09465813597082</v>
+        <v>38.09465814455221</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>15.75183325536592</v>
+        <v>15.75183317720569</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.3144623351506075</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-1.295470806548592</v>
+        <v>-1.295470806730287</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>52.06343485221353</v>
+        <v>52.06343486353902</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>7.649660555912372</v>
+        <v>7.649660582963929</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.7314484222715431</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>5.032279012327164</v>
+        <v>5.032279011245601</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>

</xml_diff>